<commit_message>
Final Game Build Milestone 1
</commit_message>
<xml_diff>
--- a/Assets/Settings/GD Elemental Game.xlsx
+++ b/Assets/Settings/GD Elemental Game.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://witscloud-my.sharepoint.com/personal/2873802_students_wits_ac_za/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GITHUB\GD LFP Group6\Assets\Settings\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6D4C3D14-E60E-40B2-AD03-2952AB842BF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2572A48B-434B-4CDB-9C71-42E6BC4A56A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{DC2CAD82-61B0-44CA-86FF-1ED257400ECA}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{DC2CAD82-61B0-44CA-86FF-1ED257400ECA}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1 (2)" sheetId="2" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="10">
   <si>
     <t>#</t>
   </si>
@@ -110,7 +111,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="32">
+  <dxfs count="21">
     <dxf>
       <fill>
         <patternFill>
@@ -286,93 +287,6 @@
             <color theme="4"/>
           </stop>
         </gradientFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <gradientFill>
-          <stop position="0">
-            <color theme="0"/>
-          </stop>
-          <stop position="1">
-            <color theme="4"/>
-          </stop>
-        </gradientFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <gradientFill degree="180">
-          <stop position="0">
-            <color theme="0"/>
-          </stop>
-          <stop position="1">
-            <color theme="4"/>
-          </stop>
-        </gradientFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="1"/>
-        </patternFill>
       </fill>
     </dxf>
   </dxfs>
@@ -704,22 +618,408 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{117CF2E8-2E02-4938-943F-AD15FA594204}">
+  <dimension ref="A1:N11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" t="s">
+        <v>0</v>
+      </c>
+      <c r="D1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F1" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1" t="s">
+        <v>2</v>
+      </c>
+      <c r="H1" t="s">
+        <v>1</v>
+      </c>
+      <c r="N1" t="str">
+        <f>_xlfn.TEXTJOIN(",",TRUE,A1:H1)</f>
+        <v>#,#,#,#,#,#,.,X</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" t="s">
+        <v>0</v>
+      </c>
+      <c r="F2" t="s">
+        <v>0</v>
+      </c>
+      <c r="G2" t="s">
+        <v>2</v>
+      </c>
+      <c r="H2" t="s">
+        <v>2</v>
+      </c>
+      <c r="N2" t="str">
+        <f t="shared" ref="N2:N11" si="0">_xlfn.TEXTJOIN(",",TRUE,A2:H2)</f>
+        <v>#,#,#,#,#,#,.,.</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" t="s">
+        <v>0</v>
+      </c>
+      <c r="C3" t="s">
+        <v>0</v>
+      </c>
+      <c r="D3" t="s">
+        <v>2</v>
+      </c>
+      <c r="E3" t="s">
+        <v>2</v>
+      </c>
+      <c r="F3" t="s">
+        <v>2</v>
+      </c>
+      <c r="G3" t="s">
+        <v>2</v>
+      </c>
+      <c r="H3" t="s">
+        <v>2</v>
+      </c>
+      <c r="N3" t="str">
+        <f t="shared" si="0"/>
+        <v>#,#,#,.,.,.,.,.</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C4" t="s">
+        <v>0</v>
+      </c>
+      <c r="D4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E4" t="s">
+        <v>2</v>
+      </c>
+      <c r="F4" t="s">
+        <v>2</v>
+      </c>
+      <c r="G4" t="s">
+        <v>5</v>
+      </c>
+      <c r="H4" t="s">
+        <v>2</v>
+      </c>
+      <c r="N4" t="str">
+        <f t="shared" si="0"/>
+        <v>#,#,#,.,.,.,F,.</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" t="s">
+        <v>9</v>
+      </c>
+      <c r="C5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D5" t="s">
+        <v>2</v>
+      </c>
+      <c r="E5" t="s">
+        <v>2</v>
+      </c>
+      <c r="F5" t="s">
+        <v>2</v>
+      </c>
+      <c r="G5" t="s">
+        <v>4</v>
+      </c>
+      <c r="H5" t="s">
+        <v>0</v>
+      </c>
+      <c r="N5" t="str">
+        <f t="shared" si="0"/>
+        <v>.,m4,.,.,.,.,m2,#</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>3</v>
+      </c>
+      <c r="B6" t="s">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>2</v>
+      </c>
+      <c r="D6" t="s">
+        <v>0</v>
+      </c>
+      <c r="E6" t="s">
+        <v>2</v>
+      </c>
+      <c r="F6" t="s">
+        <v>2</v>
+      </c>
+      <c r="G6" t="s">
+        <v>0</v>
+      </c>
+      <c r="H6" t="s">
+        <v>0</v>
+      </c>
+      <c r="N6" t="str">
+        <f t="shared" si="0"/>
+        <v>O,.,.,#,.,.,#,#</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B7" t="s">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>0</v>
+      </c>
+      <c r="D7" t="s">
+        <v>2</v>
+      </c>
+      <c r="E7" t="s">
+        <v>2</v>
+      </c>
+      <c r="F7" t="s">
+        <v>6</v>
+      </c>
+      <c r="G7" t="s">
+        <v>0</v>
+      </c>
+      <c r="H7" t="s">
+        <v>0</v>
+      </c>
+      <c r="N7" t="str">
+        <f t="shared" si="0"/>
+        <v>.,.,#,.,.,m3,#,#</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>2</v>
+      </c>
+      <c r="C8" t="s">
+        <v>0</v>
+      </c>
+      <c r="D8" t="s">
+        <v>7</v>
+      </c>
+      <c r="E8" t="s">
+        <v>2</v>
+      </c>
+      <c r="F8" t="s">
+        <v>2</v>
+      </c>
+      <c r="G8" t="s">
+        <v>0</v>
+      </c>
+      <c r="H8" t="s">
+        <v>0</v>
+      </c>
+      <c r="N8" t="str">
+        <f t="shared" si="0"/>
+        <v>m6,.,#,m6,.,.,#,#</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>0</v>
+      </c>
+      <c r="B9" t="s">
+        <v>0</v>
+      </c>
+      <c r="C9" t="s">
+        <v>0</v>
+      </c>
+      <c r="D9" t="s">
+        <v>0</v>
+      </c>
+      <c r="E9" t="s">
+        <v>2</v>
+      </c>
+      <c r="F9" t="s">
+        <v>2</v>
+      </c>
+      <c r="G9" t="s">
+        <v>0</v>
+      </c>
+      <c r="H9" t="s">
+        <v>0</v>
+      </c>
+      <c r="N9" t="str">
+        <f t="shared" si="0"/>
+        <v>#,#,#,#,.,.,#,#</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>0</v>
+      </c>
+      <c r="B10" t="s">
+        <v>0</v>
+      </c>
+      <c r="C10" t="s">
+        <v>0</v>
+      </c>
+      <c r="D10" t="s">
+        <v>2</v>
+      </c>
+      <c r="E10" t="s">
+        <v>8</v>
+      </c>
+      <c r="F10" t="s">
+        <v>2</v>
+      </c>
+      <c r="G10" t="s">
+        <v>0</v>
+      </c>
+      <c r="H10" t="s">
+        <v>0</v>
+      </c>
+      <c r="N10" t="str">
+        <f t="shared" si="0"/>
+        <v>#,#,#,.,f,.,#,#</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>0</v>
+      </c>
+      <c r="B11" t="s">
+        <v>0</v>
+      </c>
+      <c r="C11" t="s">
+        <v>0</v>
+      </c>
+      <c r="D11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E11" t="s">
+        <v>2</v>
+      </c>
+      <c r="F11" t="s">
+        <v>2</v>
+      </c>
+      <c r="G11" t="s">
+        <v>0</v>
+      </c>
+      <c r="H11" t="s">
+        <v>0</v>
+      </c>
+      <c r="N11" t="str">
+        <f t="shared" si="0"/>
+        <v>#,#,#,m6,.,.,#,#</v>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="A1:I1 K1">
+    <cfRule type="cellIs" dxfId="20" priority="8" operator="equal">
+      <formula>"O"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="19" priority="9" operator="equal">
+      <formula>"X"</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="18" priority="10" operator="containsText" text="f">
+      <formula>NOT(ISERROR(SEARCH("f",A1)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="17" priority="11" operator="containsText" text="#">
+      <formula>NOT(ISERROR(SEARCH("#",A1)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="16" priority="12" operator="containsText" text="m">
+      <formula>NOT(ISERROR(SEARCH("m",A1)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="15" priority="13" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",A1)))</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="14" priority="14" operator="equal">
+      <formula>"."</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A2:K23">
+    <cfRule type="cellIs" dxfId="13" priority="1" operator="equal">
+      <formula>"O"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="12" priority="2" operator="equal">
+      <formula>"X"</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="11" priority="3" operator="containsText" text="f">
+      <formula>NOT(ISERROR(SEARCH("f",A2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="10" priority="4" operator="containsText" text="#">
+      <formula>NOT(ISERROR(SEARCH("#",A2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="9" priority="5" operator="containsText" text="m">
+      <formula>NOT(ISERROR(SEARCH("m",A2)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="8" priority="6" operator="containsText" text="I">
+      <formula>NOT(ISERROR(SEARCH("I",A2)))</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="7" priority="7" operator="equal">
+      <formula>"."</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9BF9E27E-1378-4653-8769-0DFAA4037197}">
   <dimension ref="A1:N11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B1" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C1" t="s">
         <v>0</v>
       </c>
       <c r="D1" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E1" t="s">
         <v>0</v>
@@ -731,16 +1031,25 @@
         <v>2</v>
       </c>
       <c r="H1" t="s">
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="I1" t="s">
+        <v>2</v>
+      </c>
+      <c r="J1" t="s">
+        <v>2</v>
+      </c>
+      <c r="K1" t="s">
+        <v>0</v>
       </c>
       <c r="N1" t="str">
-        <f>_xlfn.TEXTJOIN(",",TRUE,A1:H1)</f>
-        <v>#,#,#,#,#,#,.,X</v>
+        <f>_xlfn.TEXTJOIN(",",TRUE,A1:M1)</f>
+        <v>.,.,#,.,#,#,.,#,.,.,#</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B2" t="s">
         <v>0</v>
@@ -749,10 +1058,10 @@
         <v>0</v>
       </c>
       <c r="D2" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E2" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="F2" t="s">
         <v>0</v>
@@ -761,19 +1070,28 @@
         <v>2</v>
       </c>
       <c r="H2" t="s">
+        <v>0</v>
+      </c>
+      <c r="I2" t="s">
+        <v>2</v>
+      </c>
+      <c r="J2" t="s">
+        <v>0</v>
+      </c>
+      <c r="K2" t="s">
         <v>2</v>
       </c>
       <c r="N2" t="str">
-        <f t="shared" ref="N2:N11" si="0">_xlfn.TEXTJOIN(",",TRUE,A2:H2)</f>
-        <v>#,#,#,#,#,#,.,.</v>
+        <f t="shared" ref="N2:N5" si="0">_xlfn.TEXTJOIN(",",TRUE,A2:M2)</f>
+        <v>.,#,#,.,.,#,.,#,.,#,.</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C3" t="s">
         <v>0</v>
@@ -782,7 +1100,7 @@
         <v>2</v>
       </c>
       <c r="E3" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F3" t="s">
         <v>2</v>
@@ -791,16 +1109,25 @@
         <v>2</v>
       </c>
       <c r="H3" t="s">
+        <v>0</v>
+      </c>
+      <c r="I3" t="s">
+        <v>2</v>
+      </c>
+      <c r="J3" t="s">
+        <v>0</v>
+      </c>
+      <c r="K3" t="s">
         <v>2</v>
       </c>
       <c r="N3" t="str">
         <f t="shared" si="0"/>
-        <v>#,#,#,.,.,.,.,.</v>
+        <v>O,.,#,.,#,.,.,#,.,#,.</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B4" t="s">
         <v>0</v>
@@ -812,20 +1139,29 @@
         <v>2</v>
       </c>
       <c r="E4" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F4" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G4" t="s">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="H4" t="s">
+        <v>0</v>
+      </c>
+      <c r="I4" t="s">
+        <v>2</v>
+      </c>
+      <c r="J4" t="s">
+        <v>0</v>
+      </c>
+      <c r="K4" t="s">
         <v>2</v>
       </c>
       <c r="N4" t="str">
         <f t="shared" si="0"/>
-        <v>#,#,#,.,.,.,F,.</v>
+        <v>.,#,#,.,#,#,.,#,.,#,.</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.25">
@@ -833,255 +1169,97 @@
         <v>2</v>
       </c>
       <c r="B5" t="s">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="C5" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D5" t="s">
         <v>2</v>
       </c>
       <c r="E5" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="F5" t="s">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G5" t="s">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="H5" t="s">
+        <v>0</v>
+      </c>
+      <c r="I5" t="s">
+        <v>2</v>
+      </c>
+      <c r="J5" t="s">
+        <v>2</v>
+      </c>
+      <c r="K5" t="s">
         <v>0</v>
       </c>
       <c r="N5" t="str">
         <f t="shared" si="0"/>
-        <v>.,m4,.,.,.,.,m2,#</v>
+        <v>.,.,#,.,#,#,.,#,.,.,#</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>3</v>
-      </c>
-      <c r="B6" t="s">
-        <v>2</v>
-      </c>
-      <c r="C6" t="s">
-        <v>2</v>
-      </c>
-      <c r="D6" t="s">
-        <v>0</v>
-      </c>
-      <c r="E6" t="s">
-        <v>2</v>
-      </c>
-      <c r="F6" t="s">
-        <v>2</v>
-      </c>
-      <c r="G6" t="s">
-        <v>0</v>
-      </c>
-      <c r="H6" t="s">
-        <v>0</v>
-      </c>
       <c r="N6" t="str">
-        <f t="shared" si="0"/>
-        <v>O,.,.,#,.,.,#,#</v>
+        <f t="shared" ref="N2:N11" si="1">_xlfn.TEXTJOIN(",",TRUE,A6:H6)</f>
+        <v/>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>2</v>
-      </c>
-      <c r="B7" t="s">
-        <v>2</v>
-      </c>
-      <c r="C7" t="s">
-        <v>0</v>
-      </c>
-      <c r="D7" t="s">
-        <v>2</v>
-      </c>
-      <c r="E7" t="s">
-        <v>2</v>
-      </c>
-      <c r="F7" t="s">
-        <v>6</v>
-      </c>
-      <c r="G7" t="s">
-        <v>0</v>
-      </c>
-      <c r="H7" t="s">
-        <v>0</v>
-      </c>
       <c r="N7" t="str">
-        <f t="shared" si="0"/>
-        <v>.,.,#,.,.,m3,#,#</v>
+        <f t="shared" si="1"/>
+        <v/>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>7</v>
-      </c>
-      <c r="B8" t="s">
-        <v>2</v>
-      </c>
-      <c r="C8" t="s">
-        <v>0</v>
-      </c>
-      <c r="D8" t="s">
-        <v>7</v>
-      </c>
-      <c r="E8" t="s">
-        <v>2</v>
-      </c>
-      <c r="F8" t="s">
-        <v>2</v>
-      </c>
-      <c r="G8" t="s">
-        <v>0</v>
-      </c>
-      <c r="H8" t="s">
-        <v>0</v>
-      </c>
       <c r="N8" t="str">
-        <f t="shared" si="0"/>
-        <v>m6,.,#,m6,.,.,#,#</v>
+        <f t="shared" si="1"/>
+        <v/>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>0</v>
-      </c>
-      <c r="B9" t="s">
-        <v>0</v>
-      </c>
-      <c r="C9" t="s">
-        <v>0</v>
-      </c>
-      <c r="D9" t="s">
-        <v>0</v>
-      </c>
-      <c r="E9" t="s">
-        <v>2</v>
-      </c>
-      <c r="F9" t="s">
-        <v>2</v>
-      </c>
-      <c r="G9" t="s">
-        <v>0</v>
-      </c>
-      <c r="H9" t="s">
-        <v>0</v>
-      </c>
       <c r="N9" t="str">
-        <f t="shared" si="0"/>
-        <v>#,#,#,#,.,.,#,#</v>
+        <f t="shared" si="1"/>
+        <v/>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>0</v>
-      </c>
-      <c r="B10" t="s">
-        <v>0</v>
-      </c>
-      <c r="C10" t="s">
-        <v>0</v>
-      </c>
-      <c r="D10" t="s">
-        <v>2</v>
-      </c>
-      <c r="E10" t="s">
-        <v>8</v>
-      </c>
-      <c r="F10" t="s">
-        <v>2</v>
-      </c>
-      <c r="G10" t="s">
-        <v>0</v>
-      </c>
-      <c r="H10" t="s">
-        <v>0</v>
-      </c>
       <c r="N10" t="str">
-        <f t="shared" si="0"/>
-        <v>#,#,#,.,f,.,#,#</v>
+        <f t="shared" si="1"/>
+        <v/>
       </c>
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>0</v>
-      </c>
-      <c r="B11" t="s">
-        <v>0</v>
-      </c>
-      <c r="C11" t="s">
-        <v>0</v>
-      </c>
-      <c r="D11" t="s">
-        <v>7</v>
-      </c>
-      <c r="E11" t="s">
-        <v>2</v>
-      </c>
-      <c r="F11" t="s">
-        <v>2</v>
-      </c>
-      <c r="G11" t="s">
-        <v>0</v>
-      </c>
-      <c r="H11" t="s">
-        <v>0</v>
-      </c>
       <c r="N11" t="str">
-        <f t="shared" si="0"/>
-        <v>#,#,#,m6,.,.,#,#</v>
+        <f t="shared" si="1"/>
+        <v/>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A12:K23 A9:F11 I9:K11 A2:K8 A1:I1 K1">
-    <cfRule type="cellIs" dxfId="27" priority="8" operator="equal">
+  <conditionalFormatting sqref="A1:I1 K1 A2:K23">
+    <cfRule type="cellIs" dxfId="6" priority="8" operator="equal">
       <formula>"O"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="26" priority="9" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="9" operator="equal">
       <formula>"X"</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="25" priority="11" operator="containsText" text="f">
+    <cfRule type="containsText" dxfId="4" priority="11" operator="containsText" text="f">
       <formula>NOT(ISERROR(SEARCH("f",A1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="24" priority="12" operator="containsText" text="#">
+    <cfRule type="containsText" dxfId="3" priority="12" operator="containsText" text="#">
       <formula>NOT(ISERROR(SEARCH("#",A1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="23" priority="13" operator="containsText" text="m">
+    <cfRule type="containsText" dxfId="2" priority="13" operator="containsText" text="m">
       <formula>NOT(ISERROR(SEARCH("m",A1)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="22" priority="14" operator="containsText" text="I">
+    <cfRule type="containsText" dxfId="1" priority="14" operator="containsText" text="I">
       <formula>NOT(ISERROR(SEARCH("I",A1)))</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="21" priority="15" operator="equal">
-      <formula>"."</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G9:H11">
-    <cfRule type="cellIs" dxfId="20" priority="1" operator="equal">
-      <formula>"O"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="19" priority="2" operator="equal">
-      <formula>"X"</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="18" priority="3" operator="containsText" text="f">
-      <formula>NOT(ISERROR(SEARCH("f",G9)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="17" priority="4" operator="containsText" text="#">
-      <formula>NOT(ISERROR(SEARCH("#",G9)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="16" priority="5" operator="containsText" text="m">
-      <formula>NOT(ISERROR(SEARCH("m",G9)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="15" priority="6" operator="containsText" text="I">
-      <formula>NOT(ISERROR(SEARCH("I",G9)))</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="14" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="15" operator="equal">
       <formula>"."</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Feat : Acid Detects Player
</commit_message>
<xml_diff>
--- a/Assets/Settings/GD Elemental Game.xlsx
+++ b/Assets/Settings/GD Elemental Game.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GITHUB\GD LFP Group6\Assets\Settings\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2572A48B-434B-4CDB-9C71-42E6BC4A56A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC434B45-7FC9-425D-A921-DC60108E106E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{DC2CAD82-61B0-44CA-86FF-1ED257400ECA}"/>
+    <workbookView xWindow="0" yWindow="360" windowWidth="29040" windowHeight="15720" xr2:uid="{DC2CAD82-61B0-44CA-86FF-1ED257400ECA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1 (2)" sheetId="2" r:id="rId1"/>
@@ -1013,7 +1013,7 @@
         <v>2</v>
       </c>
       <c r="B1" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="C1" t="s">
         <v>0</v>
@@ -1044,7 +1044,7 @@
       </c>
       <c r="N1" t="str">
         <f>_xlfn.TEXTJOIN(",",TRUE,A1:M1)</f>
-        <v>.,.,#,.,#,#,.,#,.,.,#</v>
+        <v>.,F,#,.,#,#,.,#,.,.,#</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
@@ -1205,7 +1205,7 @@
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="N6" t="str">
-        <f t="shared" ref="N2:N11" si="1">_xlfn.TEXTJOIN(",",TRUE,A6:H6)</f>
+        <f t="shared" ref="N6:N11" si="1">_xlfn.TEXTJOIN(",",TRUE,A6:H6)</f>
         <v/>
       </c>
     </row>

</xml_diff>